<commit_message>
correxion del formato de excel y agregado de editar y eliminacion del flaseho
</commit_message>
<xml_diff>
--- a/FORMATO.xlsx
+++ b/FORMATO.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mauro\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mauro\Downloads\control-de-clc-y-catálogos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D619D24-7961-41AF-9738-CE8642D7B73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F858BB-8330-44DB-9F00-B5A46275DBC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{83DBF909-10FB-4009-B309-0B7594E05070}"/>
+    <workbookView xWindow="0" yWindow="288" windowWidth="23232" windowHeight="12576" xr2:uid="{83DBF909-10FB-4009-B309-0B7594E05070}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="4" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">FORMATO!$A$1:$W$21</definedName>
+  </definedNames>
   <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -272,7 +275,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -723,6 +726,165 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="6"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -732,12 +894,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="16" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -748,160 +904,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="6"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -945,7 +948,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="9614086" y="21837"/>
+          <a:off x="9627421" y="25647"/>
           <a:ext cx="800100" cy="800100"/>
           <a:chOff x="0" y="0"/>
           <a:chExt cx="800100" cy="800100"/>
@@ -3064,7 +3067,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9192E898-AF1A-4EC1-B0B9-228554545DAF}">
   <dimension ref="B1:AA21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="13.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="2" style="1" customWidth="1"/>
@@ -3095,161 +3098,161 @@
     <col min="28" max="16384" width="9.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:27" ht="95.4" customHeight="1">
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
+    <row r="1" spans="2:27" ht="95.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="29"/>
+      <c r="V1" s="29"/>
+      <c r="W1" s="29"/>
       <c r="X1" s="5"/>
       <c r="AA1" s="25"/>
     </row>
-    <row r="2" spans="2:27" ht="15.75" customHeight="1">
+    <row r="2" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="5"/>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="86" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="86"/>
+      <c r="I2" s="86"/>
+      <c r="J2" s="86"/>
       <c r="K2" s="24"/>
       <c r="L2" s="5"/>
-      <c r="M2" s="36" t="s">
+      <c r="M2" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="36"/>
+      <c r="N2" s="86"/>
       <c r="O2" s="5"/>
-      <c r="P2" s="37" t="s">
+      <c r="P2" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="Q2" s="37"/>
-      <c r="R2" s="37"/>
+      <c r="Q2" s="44"/>
+      <c r="R2" s="44"/>
       <c r="S2" s="5"/>
-      <c r="T2" s="36" t="s">
+      <c r="T2" s="86" t="s">
         <v>25</v>
       </c>
-      <c r="U2" s="36"/>
-      <c r="V2" s="36"/>
-      <c r="W2" s="36"/>
+      <c r="U2" s="86"/>
+      <c r="V2" s="86"/>
+      <c r="W2" s="86"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="2:27" ht="27.75" customHeight="1">
+    <row r="3" spans="2:27" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="19"/>
-      <c r="C3" s="78" t="s">
+      <c r="C3" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="80"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="79"/>
       <c r="K3" s="23"/>
       <c r="L3" s="19"/>
-      <c r="M3" s="27" t="s">
+      <c r="M3" s="80" t="s">
         <v>29</v>
       </c>
-      <c r="N3" s="28"/>
+      <c r="N3" s="81"/>
       <c r="O3" s="10"/>
-      <c r="P3" s="32" t="s">
+      <c r="P3" s="83" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" s="33"/>
-      <c r="R3" s="34"/>
+      <c r="Q3" s="84"/>
+      <c r="R3" s="85"/>
       <c r="S3" s="10"/>
-      <c r="T3" s="29" t="s">
+      <c r="T3" s="82" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="30"/>
-      <c r="V3" s="30"/>
-      <c r="W3" s="31"/>
+      <c r="U3" s="75"/>
+      <c r="V3" s="75"/>
+      <c r="W3" s="76"/>
       <c r="X3" s="19"/>
     </row>
-    <row r="4" spans="2:27" ht="22.5" customHeight="1">
+    <row r="4" spans="2:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="10"/>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="70"/>
+      <c r="F4" s="70"/>
       <c r="G4" s="10"/>
-      <c r="H4" s="38" t="s">
+      <c r="H4" s="70" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="38"/>
-      <c r="J4" s="38"/>
-      <c r="K4" s="38"/>
-      <c r="L4" s="38"/>
-      <c r="M4" s="38"/>
-      <c r="N4" s="38"/>
-      <c r="O4" s="38"/>
-      <c r="P4" s="38"/>
-      <c r="Q4" s="38"/>
-      <c r="R4" s="38"/>
+      <c r="I4" s="70"/>
+      <c r="J4" s="70"/>
+      <c r="K4" s="70"/>
+      <c r="L4" s="70"/>
+      <c r="M4" s="70"/>
+      <c r="N4" s="70"/>
+      <c r="O4" s="70"/>
+      <c r="P4" s="70"/>
+      <c r="Q4" s="70"/>
+      <c r="R4" s="70"/>
       <c r="S4" s="10"/>
-      <c r="T4" s="38" t="s">
+      <c r="T4" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="U4" s="38"/>
-      <c r="V4" s="38"/>
-      <c r="W4" s="38"/>
+      <c r="U4" s="70"/>
+      <c r="V4" s="70"/>
+      <c r="W4" s="70"/>
       <c r="X4" s="10"/>
     </row>
-    <row r="5" spans="2:27" ht="25.5" customHeight="1">
+    <row r="5" spans="2:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="19"/>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="71" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="41"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
+      <c r="F5" s="73"/>
       <c r="G5" s="19"/>
-      <c r="H5" s="42" t="s">
+      <c r="H5" s="74" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="31"/>
+      <c r="I5" s="75"/>
+      <c r="J5" s="75"/>
+      <c r="K5" s="75"/>
+      <c r="L5" s="75"/>
+      <c r="M5" s="75"/>
+      <c r="N5" s="75"/>
+      <c r="O5" s="75"/>
+      <c r="P5" s="75"/>
+      <c r="Q5" s="75"/>
+      <c r="R5" s="76"/>
       <c r="S5" s="19"/>
-      <c r="T5" s="42" t="s">
+      <c r="T5" s="74" t="s">
         <v>34</v>
       </c>
-      <c r="U5" s="30"/>
-      <c r="V5" s="30"/>
-      <c r="W5" s="31"/>
+      <c r="U5" s="75"/>
+      <c r="V5" s="75"/>
+      <c r="W5" s="76"/>
       <c r="X5" s="19"/>
     </row>
-    <row r="6" spans="2:27" ht="17.25" customHeight="1">
+    <row r="6" spans="2:27" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="19"/>
       <c r="C6" s="19"/>
       <c r="D6" s="19"/>
@@ -3274,149 +3277,149 @@
       <c r="W6" s="19"/>
       <c r="X6" s="19"/>
     </row>
-    <row r="7" spans="2:27" ht="12.75" customHeight="1">
+    <row r="7" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="19"/>
-      <c r="C7" s="81" t="s">
+      <c r="C7" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="59"/>
-      <c r="E7" s="84" t="s">
+      <c r="D7" s="55"/>
+      <c r="E7" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="85"/>
-      <c r="G7" s="85"/>
-      <c r="H7" s="85"/>
-      <c r="I7" s="85"/>
-      <c r="J7" s="85"/>
-      <c r="K7" s="85"/>
-      <c r="L7" s="85"/>
-      <c r="M7" s="86"/>
-      <c r="N7" s="49" t="s">
+      <c r="F7" s="52"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="52"/>
+      <c r="L7" s="52"/>
+      <c r="M7" s="53"/>
+      <c r="N7" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="50"/>
-      <c r="P7" s="51"/>
-      <c r="Q7" s="47" t="s">
+      <c r="O7" s="60"/>
+      <c r="P7" s="61"/>
+      <c r="Q7" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="R7" s="47" t="s">
+      <c r="R7" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="S7" s="58" t="s">
+      <c r="S7" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="T7" s="59"/>
-      <c r="U7" s="47" t="s">
+      <c r="T7" s="55"/>
+      <c r="U7" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="V7" s="47" t="s">
+      <c r="V7" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="W7" s="47" t="s">
+      <c r="W7" s="49" t="s">
         <v>12</v>
       </c>
       <c r="X7" s="19"/>
     </row>
-    <row r="8" spans="2:27" ht="15" customHeight="1">
+    <row r="8" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="10"/>
-      <c r="C8" s="60"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="82" t="s">
+      <c r="C8" s="57"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="82" t="s">
+      <c r="F8" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="84" t="s">
+      <c r="G8" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="85"/>
-      <c r="I8" s="85"/>
-      <c r="J8" s="85"/>
-      <c r="K8" s="85"/>
-      <c r="L8" s="85"/>
-      <c r="M8" s="86"/>
-      <c r="N8" s="52"/>
-      <c r="O8" s="53"/>
-      <c r="P8" s="54"/>
-      <c r="Q8" s="48"/>
-      <c r="R8" s="48"/>
-      <c r="S8" s="60"/>
-      <c r="T8" s="61"/>
-      <c r="U8" s="48"/>
-      <c r="V8" s="48"/>
-      <c r="W8" s="48"/>
+      <c r="H8" s="52"/>
+      <c r="I8" s="52"/>
+      <c r="J8" s="52"/>
+      <c r="K8" s="52"/>
+      <c r="L8" s="52"/>
+      <c r="M8" s="53"/>
+      <c r="N8" s="62"/>
+      <c r="O8" s="63"/>
+      <c r="P8" s="64"/>
+      <c r="Q8" s="50"/>
+      <c r="R8" s="50"/>
+      <c r="S8" s="57"/>
+      <c r="T8" s="58"/>
+      <c r="U8" s="50"/>
+      <c r="V8" s="50"/>
+      <c r="W8" s="50"/>
       <c r="X8" s="10"/>
     </row>
-    <row r="9" spans="2:27" ht="20.25" customHeight="1">
+    <row r="9" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="19"/>
-      <c r="C9" s="60"/>
-      <c r="D9" s="61"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="58"/>
       <c r="E9" s="26" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="81" t="s">
+      <c r="G9" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="59"/>
-      <c r="I9" s="81" t="s">
+      <c r="H9" s="55"/>
+      <c r="I9" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="J9" s="83"/>
-      <c r="K9" s="83"/>
-      <c r="L9" s="83"/>
-      <c r="M9" s="59"/>
-      <c r="N9" s="55"/>
-      <c r="O9" s="56"/>
-      <c r="P9" s="57"/>
-      <c r="Q9" s="48"/>
-      <c r="R9" s="48"/>
-      <c r="S9" s="60"/>
-      <c r="T9" s="61"/>
-      <c r="U9" s="48"/>
-      <c r="V9" s="48"/>
-      <c r="W9" s="48"/>
+      <c r="J9" s="56"/>
+      <c r="K9" s="56"/>
+      <c r="L9" s="56"/>
+      <c r="M9" s="55"/>
+      <c r="N9" s="65"/>
+      <c r="O9" s="66"/>
+      <c r="P9" s="67"/>
+      <c r="Q9" s="50"/>
+      <c r="R9" s="50"/>
+      <c r="S9" s="57"/>
+      <c r="T9" s="58"/>
+      <c r="U9" s="50"/>
+      <c r="V9" s="50"/>
+      <c r="W9" s="50"/>
       <c r="X9" s="19"/>
     </row>
-    <row r="10" spans="2:27" ht="59.25" customHeight="1">
+    <row r="10" spans="2:27" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="19"/>
-      <c r="C10" s="62">
+      <c r="C10" s="69">
         <v>4446</v>
       </c>
-      <c r="D10" s="62"/>
+      <c r="D10" s="69"/>
       <c r="E10" s="22" t="s">
         <v>35</v>
       </c>
       <c r="F10" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="63" t="s">
+      <c r="G10" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="H10" s="63"/>
-      <c r="I10" s="63" t="s">
+      <c r="H10" s="36"/>
+      <c r="I10" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="63"/>
-      <c r="K10" s="63"/>
-      <c r="L10" s="63"/>
-      <c r="M10" s="63"/>
-      <c r="N10" s="64" t="s">
+      <c r="J10" s="36"/>
+      <c r="K10" s="36"/>
+      <c r="L10" s="36"/>
+      <c r="M10" s="36"/>
+      <c r="N10" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="O10" s="65"/>
-      <c r="P10" s="66"/>
+      <c r="O10" s="38"/>
+      <c r="P10" s="39"/>
       <c r="Q10" s="21"/>
       <c r="R10" s="20">
         <v>1</v>
       </c>
-      <c r="S10" s="67">
+      <c r="S10" s="40">
         <v>0</v>
       </c>
-      <c r="T10" s="68"/>
+      <c r="T10" s="41"/>
       <c r="U10" s="20">
         <v>0.16</v>
       </c>
@@ -3429,39 +3432,39 @@
       </c>
       <c r="X10" s="19"/>
     </row>
-    <row r="11" spans="2:27" s="14" customFormat="1" ht="48.75" customHeight="1">
+    <row r="11" spans="2:27" s="14" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="10"/>
-      <c r="C11" s="43" t="s">
+      <c r="C11" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
-      <c r="H11" s="44"/>
-      <c r="I11" s="44"/>
-      <c r="J11" s="44"/>
-      <c r="K11" s="44"/>
-      <c r="L11" s="44"/>
-      <c r="M11" s="44"/>
-      <c r="N11" s="44"/>
-      <c r="O11" s="44"/>
-      <c r="P11" s="44"/>
-      <c r="Q11" s="44"/>
-      <c r="R11" s="44"/>
-      <c r="S11" s="45"/>
-      <c r="T11" s="46" t="s">
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
+      <c r="I11" s="46"/>
+      <c r="J11" s="46"/>
+      <c r="K11" s="46"/>
+      <c r="L11" s="46"/>
+      <c r="M11" s="46"/>
+      <c r="N11" s="46"/>
+      <c r="O11" s="46"/>
+      <c r="P11" s="46"/>
+      <c r="Q11" s="46"/>
+      <c r="R11" s="46"/>
+      <c r="S11" s="47"/>
+      <c r="T11" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="U11" s="46"/>
-      <c r="V11" s="46"/>
+      <c r="U11" s="48"/>
+      <c r="V11" s="48"/>
       <c r="W11" s="15">
         <f>SUM(W10:W10)</f>
         <v>1.1599999999999999</v>
       </c>
       <c r="X11" s="10"/>
     </row>
-    <row r="12" spans="2:27" s="14" customFormat="1" ht="14.25" customHeight="1">
+    <row r="12" spans="2:27" s="14" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="10"/>
       <c r="C12" s="18"/>
       <c r="D12" s="18"/>
@@ -3486,59 +3489,59 @@
       <c r="W12" s="15"/>
       <c r="X12" s="10"/>
     </row>
-    <row r="13" spans="2:27" ht="12" customHeight="1">
-      <c r="C13" s="76"/>
-      <c r="D13" s="77"/>
-      <c r="E13" s="77"/>
-      <c r="F13" s="77"/>
-      <c r="G13" s="77"/>
-      <c r="H13" s="77"/>
-      <c r="I13" s="77"/>
-      <c r="J13" s="77"/>
-      <c r="K13" s="77"/>
-      <c r="L13" s="77"/>
-      <c r="M13" s="77"/>
-      <c r="N13" s="77"/>
-      <c r="O13" s="77"/>
-      <c r="P13" s="77"/>
-      <c r="Q13" s="77"/>
-      <c r="R13" s="77"/>
-      <c r="S13" s="77"/>
-      <c r="T13" s="77"/>
-      <c r="U13" s="77"/>
-      <c r="V13" s="77"/>
-      <c r="W13" s="77"/>
+    <row r="13" spans="2:27" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="30"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="31"/>
+      <c r="O13" s="31"/>
+      <c r="P13" s="31"/>
+      <c r="Q13" s="31"/>
+      <c r="R13" s="31"/>
+      <c r="S13" s="31"/>
+      <c r="T13" s="31"/>
+      <c r="U13" s="31"/>
+      <c r="V13" s="31"/>
+      <c r="W13" s="31"/>
       <c r="X13" s="4"/>
-      <c r="Y13" s="69"/>
-      <c r="Z13" s="69"/>
+      <c r="Y13" s="42"/>
+      <c r="Z13" s="42"/>
     </row>
-    <row r="14" spans="2:27" ht="12.75" customHeight="1">
-      <c r="C14" s="70" t="s">
+    <row r="14" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="37"/>
-      <c r="I14" s="37"/>
-      <c r="L14" s="70" t="s">
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="L14" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="M14" s="37"/>
-      <c r="N14" s="37"/>
-      <c r="O14" s="37"/>
-      <c r="P14" s="37"/>
-      <c r="R14" s="70" t="s">
+      <c r="M14" s="44"/>
+      <c r="N14" s="44"/>
+      <c r="O14" s="44"/>
+      <c r="P14" s="44"/>
+      <c r="R14" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="S14" s="37"/>
-      <c r="T14" s="37"/>
-      <c r="U14" s="37"/>
-      <c r="V14" s="37"/>
-      <c r="W14" s="37"/>
+      <c r="S14" s="44"/>
+      <c r="T14" s="44"/>
+      <c r="U14" s="44"/>
+      <c r="V14" s="44"/>
+      <c r="W14" s="44"/>
     </row>
-    <row r="15" spans="2:27" ht="76.5" customHeight="1">
+    <row r="15" spans="2:27" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="13" t="s">
         <v>41</v>
       </c>
@@ -3550,54 +3553,54 @@
       <c r="I15" s="13"/>
       <c r="J15" s="12"/>
       <c r="K15" s="9"/>
-      <c r="L15" s="71" t="s">
+      <c r="L15" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="M15" s="71"/>
-      <c r="N15" s="71"/>
-      <c r="O15" s="71"/>
-      <c r="P15" s="71"/>
+      <c r="M15" s="32"/>
+      <c r="N15" s="32"/>
+      <c r="O15" s="32"/>
+      <c r="P15" s="32"/>
       <c r="Q15" s="11"/>
-      <c r="R15" s="72" t="s">
+      <c r="R15" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="S15" s="72"/>
-      <c r="T15" s="72"/>
-      <c r="U15" s="72"/>
-      <c r="V15" s="72"/>
-      <c r="W15" s="72"/>
+      <c r="S15" s="33"/>
+      <c r="T15" s="33"/>
+      <c r="U15" s="33"/>
+      <c r="V15" s="33"/>
+      <c r="W15" s="33"/>
     </row>
-    <row r="16" spans="2:27" ht="25.5" customHeight="1">
+    <row r="16" spans="2:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="10"/>
-      <c r="C16" s="73" t="s">
+      <c r="C16" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="73"/>
-      <c r="E16" s="73"/>
-      <c r="F16" s="73"/>
-      <c r="G16" s="73"/>
-      <c r="H16" s="73"/>
-      <c r="I16" s="73"/>
-      <c r="J16" s="73"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="34"/>
+      <c r="J16" s="34"/>
       <c r="K16" s="9"/>
-      <c r="L16" s="73" t="s">
+      <c r="L16" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="M16" s="74"/>
-      <c r="N16" s="74"/>
-      <c r="O16" s="74"/>
-      <c r="P16" s="74"/>
+      <c r="M16" s="35"/>
+      <c r="N16" s="35"/>
+      <c r="O16" s="35"/>
+      <c r="P16" s="35"/>
       <c r="Q16" s="7"/>
-      <c r="R16" s="74" t="s">
+      <c r="R16" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="S16" s="74"/>
-      <c r="T16" s="74"/>
-      <c r="U16" s="74"/>
-      <c r="V16" s="74"/>
-      <c r="W16" s="74"/>
+      <c r="S16" s="35"/>
+      <c r="T16" s="35"/>
+      <c r="U16" s="35"/>
+      <c r="V16" s="35"/>
+      <c r="W16" s="35"/>
     </row>
-    <row r="17" spans="2:24" ht="25.5" customHeight="1">
+    <row r="17" spans="2:24" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="10"/>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
@@ -3621,7 +3624,7 @@
       <c r="V17" s="6"/>
       <c r="W17" s="6"/>
     </row>
-    <row r="18" spans="2:24" ht="12.75" customHeight="1">
+    <row r="18" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="10"/>
       <c r="C18" s="8"/>
       <c r="D18" s="6"/>
@@ -3645,34 +3648,34 @@
       <c r="V18" s="6"/>
       <c r="W18" s="6"/>
     </row>
-    <row r="19" spans="2:24" ht="57" customHeight="1">
+    <row r="19" spans="2:24" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="4"/>
-      <c r="C19" s="75" t="s">
+      <c r="C19" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="35"/>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
-      <c r="J19" s="35"/>
-      <c r="K19" s="35"/>
-      <c r="L19" s="35"/>
-      <c r="M19" s="35"/>
-      <c r="N19" s="35"/>
-      <c r="O19" s="35"/>
-      <c r="P19" s="35"/>
-      <c r="Q19" s="35"/>
-      <c r="R19" s="35"/>
-      <c r="S19" s="35"/>
-      <c r="T19" s="35"/>
-      <c r="U19" s="35"/>
-      <c r="V19" s="35"/>
-      <c r="W19" s="35"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
+      <c r="J19" s="29"/>
+      <c r="K19" s="29"/>
+      <c r="L19" s="29"/>
+      <c r="M19" s="29"/>
+      <c r="N19" s="29"/>
+      <c r="O19" s="29"/>
+      <c r="P19" s="29"/>
+      <c r="Q19" s="29"/>
+      <c r="R19" s="29"/>
+      <c r="S19" s="29"/>
+      <c r="T19" s="29"/>
+      <c r="U19" s="29"/>
+      <c r="V19" s="29"/>
+      <c r="W19" s="29"/>
       <c r="X19" s="4"/>
     </row>
-    <row r="21" spans="2:24">
+    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
       <c r="C21" s="3"/>
       <c r="E21" s="2">
         <v>46176.954704459997</v>
@@ -3680,13 +3683,33 @@
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="C19:W19"/>
-    <mergeCell ref="C13:W13"/>
-    <mergeCell ref="L15:P15"/>
-    <mergeCell ref="R15:W15"/>
-    <mergeCell ref="C16:J16"/>
-    <mergeCell ref="L16:P16"/>
-    <mergeCell ref="R16:W16"/>
+    <mergeCell ref="C3:J3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="T3:W3"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="B1:W1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="T2:W2"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="H4:R4"/>
+    <mergeCell ref="T4:W4"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="H5:R5"/>
+    <mergeCell ref="T5:W5"/>
+    <mergeCell ref="C7:D9"/>
+    <mergeCell ref="E7:M7"/>
+    <mergeCell ref="N7:P9"/>
+    <mergeCell ref="Q7:Q9"/>
+    <mergeCell ref="R7:R9"/>
+    <mergeCell ref="U7:U9"/>
+    <mergeCell ref="V7:V9"/>
+    <mergeCell ref="W7:W9"/>
+    <mergeCell ref="G8:M8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="I9:M9"/>
+    <mergeCell ref="S7:T9"/>
     <mergeCell ref="I10:M10"/>
     <mergeCell ref="N10:P10"/>
     <mergeCell ref="S10:T10"/>
@@ -3696,38 +3719,21 @@
     <mergeCell ref="R14:W14"/>
     <mergeCell ref="C11:S11"/>
     <mergeCell ref="T11:V11"/>
-    <mergeCell ref="U7:U9"/>
-    <mergeCell ref="V7:V9"/>
-    <mergeCell ref="W7:W9"/>
-    <mergeCell ref="G8:M8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:M9"/>
-    <mergeCell ref="C7:D9"/>
-    <mergeCell ref="E7:M7"/>
-    <mergeCell ref="N7:P9"/>
-    <mergeCell ref="Q7:Q9"/>
-    <mergeCell ref="R7:R9"/>
-    <mergeCell ref="S7:T9"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="G10:H10"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="H4:R4"/>
-    <mergeCell ref="T4:W4"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="H5:R5"/>
-    <mergeCell ref="T5:W5"/>
-    <mergeCell ref="C3:J3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="T3:W3"/>
-    <mergeCell ref="P3:R3"/>
-    <mergeCell ref="B1:W1"/>
-    <mergeCell ref="C2:J2"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="T2:W2"/>
+    <mergeCell ref="C19:W19"/>
+    <mergeCell ref="C13:W13"/>
+    <mergeCell ref="L15:P15"/>
+    <mergeCell ref="R15:W15"/>
+    <mergeCell ref="C16:J16"/>
+    <mergeCell ref="L16:P16"/>
+    <mergeCell ref="R16:W16"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="80" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="74" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <colBreaks count="1" manualBreakCount="1">
+    <brk id="23" max="1048575" man="1"/>
+  </colBreaks>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
buscar numero de cuenta y agregar cosas desde ahi
</commit_message>
<xml_diff>
--- a/FORMATO.xlsx
+++ b/FORMATO.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F858BB-8330-44DB-9F00-B5A46275DBC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="288" windowWidth="23232" windowHeight="12576" xr2:uid="{83DBF909-10FB-4009-B309-0B7594E05070}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{83DBF909-10FB-4009-B309-0B7594E05070}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="4" r:id="rId1"/>
@@ -275,7 +275,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -729,12 +729,165 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="6"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -751,159 +904,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="6"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -948,7 +948,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="9627421" y="25647"/>
+          <a:off x="9614086" y="21837"/>
           <a:ext cx="800100" cy="800100"/>
           <a:chOff x="0" y="0"/>
           <a:chExt cx="800100" cy="800100"/>
@@ -3067,7 +3067,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9192E898-AF1A-4EC1-B0B9-228554545DAF}">
   <dimension ref="B1:AA21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="2.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="2" style="1" customWidth="1"/>
@@ -3098,161 +3098,161 @@
     <col min="28" max="16384" width="9.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:27" ht="95.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
-      <c r="S1" s="29"/>
-      <c r="T1" s="29"/>
-      <c r="U1" s="29"/>
-      <c r="V1" s="29"/>
-      <c r="W1" s="29"/>
+    <row r="1" spans="2:27" ht="95.4" customHeight="1">
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="39"/>
+      <c r="U1" s="39"/>
+      <c r="V1" s="39"/>
+      <c r="W1" s="39"/>
       <c r="X1" s="5"/>
       <c r="AA1" s="25"/>
     </row>
-    <row r="2" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:27" ht="15.75" customHeight="1">
       <c r="B2" s="5"/>
-      <c r="C2" s="86" t="s">
+      <c r="C2" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
       <c r="K2" s="24"/>
       <c r="L2" s="5"/>
-      <c r="M2" s="86" t="s">
+      <c r="M2" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="86"/>
+      <c r="N2" s="40"/>
       <c r="O2" s="5"/>
-      <c r="P2" s="44" t="s">
+      <c r="P2" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="Q2" s="44"/>
-      <c r="R2" s="44"/>
+      <c r="Q2" s="41"/>
+      <c r="R2" s="41"/>
       <c r="S2" s="5"/>
-      <c r="T2" s="86" t="s">
+      <c r="T2" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="U2" s="86"/>
-      <c r="V2" s="86"/>
-      <c r="W2" s="86"/>
+      <c r="U2" s="40"/>
+      <c r="V2" s="40"/>
+      <c r="W2" s="40"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="2:27" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:27" ht="27.75" customHeight="1">
       <c r="B3" s="19"/>
-      <c r="C3" s="77" t="s">
+      <c r="C3" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="78"/>
-      <c r="E3" s="78"/>
-      <c r="F3" s="78"/>
-      <c r="G3" s="78"/>
-      <c r="H3" s="78"/>
-      <c r="I3" s="78"/>
-      <c r="J3" s="79"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="30"/>
       <c r="K3" s="23"/>
       <c r="L3" s="19"/>
-      <c r="M3" s="80" t="s">
+      <c r="M3" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="N3" s="81"/>
+      <c r="N3" s="32"/>
       <c r="O3" s="10"/>
-      <c r="P3" s="83" t="s">
+      <c r="P3" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" s="84"/>
-      <c r="R3" s="85"/>
+      <c r="Q3" s="37"/>
+      <c r="R3" s="38"/>
       <c r="S3" s="10"/>
-      <c r="T3" s="82" t="s">
+      <c r="T3" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="75"/>
-      <c r="V3" s="75"/>
-      <c r="W3" s="76"/>
+      <c r="U3" s="34"/>
+      <c r="V3" s="34"/>
+      <c r="W3" s="35"/>
       <c r="X3" s="19"/>
     </row>
-    <row r="4" spans="2:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:27" ht="22.5" customHeight="1">
       <c r="B4" s="10"/>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
       <c r="G4" s="10"/>
-      <c r="H4" s="70" t="s">
+      <c r="H4" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="70"/>
-      <c r="J4" s="70"/>
-      <c r="K4" s="70"/>
-      <c r="L4" s="70"/>
-      <c r="M4" s="70"/>
-      <c r="N4" s="70"/>
-      <c r="O4" s="70"/>
-      <c r="P4" s="70"/>
-      <c r="Q4" s="70"/>
-      <c r="R4" s="70"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
+      <c r="K4" s="42"/>
+      <c r="L4" s="42"/>
+      <c r="M4" s="42"/>
+      <c r="N4" s="42"/>
+      <c r="O4" s="42"/>
+      <c r="P4" s="42"/>
+      <c r="Q4" s="42"/>
+      <c r="R4" s="42"/>
       <c r="S4" s="10"/>
-      <c r="T4" s="70" t="s">
+      <c r="T4" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="U4" s="70"/>
-      <c r="V4" s="70"/>
-      <c r="W4" s="70"/>
+      <c r="U4" s="42"/>
+      <c r="V4" s="42"/>
+      <c r="W4" s="42"/>
       <c r="X4" s="10"/>
     </row>
-    <row r="5" spans="2:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:27" ht="25.5" customHeight="1">
       <c r="B5" s="19"/>
-      <c r="C5" s="71" t="s">
+      <c r="C5" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="72"/>
-      <c r="E5" s="72"/>
-      <c r="F5" s="73"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="45"/>
       <c r="G5" s="19"/>
-      <c r="H5" s="74" t="s">
+      <c r="H5" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="75"/>
-      <c r="J5" s="75"/>
-      <c r="K5" s="75"/>
-      <c r="L5" s="75"/>
-      <c r="M5" s="75"/>
-      <c r="N5" s="75"/>
-      <c r="O5" s="75"/>
-      <c r="P5" s="75"/>
-      <c r="Q5" s="75"/>
-      <c r="R5" s="76"/>
+      <c r="I5" s="34"/>
+      <c r="J5" s="34"/>
+      <c r="K5" s="34"/>
+      <c r="L5" s="34"/>
+      <c r="M5" s="34"/>
+      <c r="N5" s="34"/>
+      <c r="O5" s="34"/>
+      <c r="P5" s="34"/>
+      <c r="Q5" s="34"/>
+      <c r="R5" s="35"/>
       <c r="S5" s="19"/>
-      <c r="T5" s="74" t="s">
+      <c r="T5" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="U5" s="75"/>
-      <c r="V5" s="75"/>
-      <c r="W5" s="76"/>
+      <c r="U5" s="34"/>
+      <c r="V5" s="34"/>
+      <c r="W5" s="35"/>
       <c r="X5" s="19"/>
     </row>
-    <row r="6" spans="2:27" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:27" ht="17.25" customHeight="1">
       <c r="B6" s="19"/>
       <c r="C6" s="19"/>
       <c r="D6" s="19"/>
@@ -3277,12 +3277,12 @@
       <c r="W6" s="19"/>
       <c r="X6" s="19"/>
     </row>
-    <row r="7" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:27" ht="12.75" customHeight="1">
       <c r="B7" s="19"/>
-      <c r="C7" s="54" t="s">
+      <c r="C7" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="55"/>
+      <c r="D7" s="48"/>
       <c r="E7" s="51" t="s">
         <v>19</v>
       </c>
@@ -3294,36 +3294,36 @@
       <c r="K7" s="52"/>
       <c r="L7" s="52"/>
       <c r="M7" s="53"/>
-      <c r="N7" s="59" t="s">
+      <c r="N7" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="60"/>
-      <c r="P7" s="61"/>
-      <c r="Q7" s="49" t="s">
+      <c r="O7" s="55"/>
+      <c r="P7" s="56"/>
+      <c r="Q7" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="R7" s="49" t="s">
+      <c r="R7" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="S7" s="68" t="s">
+      <c r="S7" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="T7" s="55"/>
-      <c r="U7" s="49" t="s">
+      <c r="T7" s="48"/>
+      <c r="U7" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="V7" s="49" t="s">
+      <c r="V7" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="W7" s="49" t="s">
+      <c r="W7" s="63" t="s">
         <v>12</v>
       </c>
       <c r="X7" s="19"/>
     </row>
-    <row r="8" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:27" ht="15" customHeight="1">
       <c r="B8" s="10"/>
-      <c r="C8" s="57"/>
-      <c r="D8" s="58"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="50"/>
       <c r="E8" s="27" t="s">
         <v>11</v>
       </c>
@@ -3339,87 +3339,87 @@
       <c r="K8" s="52"/>
       <c r="L8" s="52"/>
       <c r="M8" s="53"/>
-      <c r="N8" s="62"/>
-      <c r="O8" s="63"/>
-      <c r="P8" s="64"/>
-      <c r="Q8" s="50"/>
-      <c r="R8" s="50"/>
-      <c r="S8" s="57"/>
-      <c r="T8" s="58"/>
-      <c r="U8" s="50"/>
-      <c r="V8" s="50"/>
-      <c r="W8" s="50"/>
+      <c r="N8" s="57"/>
+      <c r="O8" s="58"/>
+      <c r="P8" s="59"/>
+      <c r="Q8" s="64"/>
+      <c r="R8" s="64"/>
+      <c r="S8" s="49"/>
+      <c r="T8" s="50"/>
+      <c r="U8" s="64"/>
+      <c r="V8" s="64"/>
+      <c r="W8" s="64"/>
       <c r="X8" s="10"/>
     </row>
-    <row r="9" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:27" ht="20.25" customHeight="1">
       <c r="B9" s="19"/>
-      <c r="C9" s="57"/>
-      <c r="D9" s="58"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="50"/>
       <c r="E9" s="26" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="54" t="s">
+      <c r="G9" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="55"/>
-      <c r="I9" s="54" t="s">
+      <c r="H9" s="48"/>
+      <c r="I9" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="J9" s="56"/>
-      <c r="K9" s="56"/>
-      <c r="L9" s="56"/>
-      <c r="M9" s="55"/>
-      <c r="N9" s="65"/>
-      <c r="O9" s="66"/>
-      <c r="P9" s="67"/>
-      <c r="Q9" s="50"/>
-      <c r="R9" s="50"/>
-      <c r="S9" s="57"/>
-      <c r="T9" s="58"/>
-      <c r="U9" s="50"/>
-      <c r="V9" s="50"/>
-      <c r="W9" s="50"/>
+      <c r="J9" s="65"/>
+      <c r="K9" s="65"/>
+      <c r="L9" s="65"/>
+      <c r="M9" s="48"/>
+      <c r="N9" s="60"/>
+      <c r="O9" s="61"/>
+      <c r="P9" s="62"/>
+      <c r="Q9" s="64"/>
+      <c r="R9" s="64"/>
+      <c r="S9" s="49"/>
+      <c r="T9" s="50"/>
+      <c r="U9" s="64"/>
+      <c r="V9" s="64"/>
+      <c r="W9" s="64"/>
       <c r="X9" s="19"/>
     </row>
-    <row r="10" spans="2:27" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:27" ht="59.25" customHeight="1">
       <c r="B10" s="19"/>
-      <c r="C10" s="69">
+      <c r="C10" s="79">
         <v>4446</v>
       </c>
-      <c r="D10" s="69"/>
+      <c r="D10" s="79"/>
       <c r="E10" s="22" t="s">
         <v>35</v>
       </c>
       <c r="F10" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="36" t="s">
+      <c r="G10" s="67" t="s">
         <v>37</v>
       </c>
-      <c r="H10" s="36"/>
-      <c r="I10" s="36" t="s">
+      <c r="H10" s="67"/>
+      <c r="I10" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="36"/>
-      <c r="K10" s="36"/>
-      <c r="L10" s="36"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="37" t="s">
+      <c r="J10" s="67"/>
+      <c r="K10" s="67"/>
+      <c r="L10" s="67"/>
+      <c r="M10" s="67"/>
+      <c r="N10" s="68" t="s">
         <v>39</v>
       </c>
-      <c r="O10" s="38"/>
-      <c r="P10" s="39"/>
+      <c r="O10" s="69"/>
+      <c r="P10" s="70"/>
       <c r="Q10" s="21"/>
       <c r="R10" s="20">
         <v>1</v>
       </c>
-      <c r="S10" s="40">
+      <c r="S10" s="71">
         <v>0</v>
       </c>
-      <c r="T10" s="41"/>
+      <c r="T10" s="72"/>
       <c r="U10" s="20">
         <v>0.16</v>
       </c>
@@ -3432,39 +3432,39 @@
       </c>
       <c r="X10" s="19"/>
     </row>
-    <row r="11" spans="2:27" s="14" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:27" s="14" customFormat="1" ht="48.75" customHeight="1">
       <c r="B11" s="10"/>
-      <c r="C11" s="45" t="s">
+      <c r="C11" s="75" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46"/>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="46"/>
-      <c r="I11" s="46"/>
-      <c r="J11" s="46"/>
-      <c r="K11" s="46"/>
-      <c r="L11" s="46"/>
-      <c r="M11" s="46"/>
-      <c r="N11" s="46"/>
-      <c r="O11" s="46"/>
-      <c r="P11" s="46"/>
-      <c r="Q11" s="46"/>
-      <c r="R11" s="46"/>
-      <c r="S11" s="47"/>
-      <c r="T11" s="48" t="s">
+      <c r="D11" s="76"/>
+      <c r="E11" s="76"/>
+      <c r="F11" s="76"/>
+      <c r="G11" s="76"/>
+      <c r="H11" s="76"/>
+      <c r="I11" s="76"/>
+      <c r="J11" s="76"/>
+      <c r="K11" s="76"/>
+      <c r="L11" s="76"/>
+      <c r="M11" s="76"/>
+      <c r="N11" s="76"/>
+      <c r="O11" s="76"/>
+      <c r="P11" s="76"/>
+      <c r="Q11" s="76"/>
+      <c r="R11" s="76"/>
+      <c r="S11" s="77"/>
+      <c r="T11" s="78" t="s">
         <v>6</v>
       </c>
-      <c r="U11" s="48"/>
-      <c r="V11" s="48"/>
+      <c r="U11" s="78"/>
+      <c r="V11" s="78"/>
       <c r="W11" s="15">
         <f>SUM(W10:W10)</f>
         <v>1.1599999999999999</v>
       </c>
       <c r="X11" s="10"/>
     </row>
-    <row r="12" spans="2:27" s="14" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:27" s="14" customFormat="1" ht="14.25" customHeight="1">
       <c r="B12" s="10"/>
       <c r="C12" s="18"/>
       <c r="D12" s="18"/>
@@ -3489,59 +3489,59 @@
       <c r="W12" s="15"/>
       <c r="X12" s="10"/>
     </row>
-    <row r="13" spans="2:27" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="30"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="31"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="31"/>
-      <c r="I13" s="31"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="31"/>
-      <c r="L13" s="31"/>
-      <c r="M13" s="31"/>
-      <c r="N13" s="31"/>
-      <c r="O13" s="31"/>
-      <c r="P13" s="31"/>
-      <c r="Q13" s="31"/>
-      <c r="R13" s="31"/>
-      <c r="S13" s="31"/>
-      <c r="T13" s="31"/>
-      <c r="U13" s="31"/>
-      <c r="V13" s="31"/>
-      <c r="W13" s="31"/>
+    <row r="13" spans="2:27" ht="12" customHeight="1">
+      <c r="C13" s="81"/>
+      <c r="D13" s="82"/>
+      <c r="E13" s="82"/>
+      <c r="F13" s="82"/>
+      <c r="G13" s="82"/>
+      <c r="H13" s="82"/>
+      <c r="I13" s="82"/>
+      <c r="J13" s="82"/>
+      <c r="K13" s="82"/>
+      <c r="L13" s="82"/>
+      <c r="M13" s="82"/>
+      <c r="N13" s="82"/>
+      <c r="O13" s="82"/>
+      <c r="P13" s="82"/>
+      <c r="Q13" s="82"/>
+      <c r="R13" s="82"/>
+      <c r="S13" s="82"/>
+      <c r="T13" s="82"/>
+      <c r="U13" s="82"/>
+      <c r="V13" s="82"/>
+      <c r="W13" s="82"/>
       <c r="X13" s="4"/>
-      <c r="Y13" s="42"/>
-      <c r="Z13" s="42"/>
+      <c r="Y13" s="73"/>
+      <c r="Z13" s="73"/>
     </row>
-    <row r="14" spans="2:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="43" t="s">
+    <row r="14" spans="2:27" ht="12.75" customHeight="1">
+      <c r="C14" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="44"/>
-      <c r="L14" s="43" t="s">
+      <c r="D14" s="41"/>
+      <c r="E14" s="41"/>
+      <c r="F14" s="41"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="41"/>
+      <c r="I14" s="41"/>
+      <c r="L14" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="M14" s="44"/>
-      <c r="N14" s="44"/>
-      <c r="O14" s="44"/>
-      <c r="P14" s="44"/>
-      <c r="R14" s="43" t="s">
+      <c r="M14" s="41"/>
+      <c r="N14" s="41"/>
+      <c r="O14" s="41"/>
+      <c r="P14" s="41"/>
+      <c r="R14" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="S14" s="44"/>
-      <c r="T14" s="44"/>
-      <c r="U14" s="44"/>
-      <c r="V14" s="44"/>
-      <c r="W14" s="44"/>
+      <c r="S14" s="41"/>
+      <c r="T14" s="41"/>
+      <c r="U14" s="41"/>
+      <c r="V14" s="41"/>
+      <c r="W14" s="41"/>
     </row>
-    <row r="15" spans="2:27" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:27" ht="76.5" customHeight="1">
       <c r="C15" s="13" t="s">
         <v>41</v>
       </c>
@@ -3553,54 +3553,54 @@
       <c r="I15" s="13"/>
       <c r="J15" s="12"/>
       <c r="K15" s="9"/>
-      <c r="L15" s="32" t="s">
+      <c r="L15" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="M15" s="32"/>
-      <c r="N15" s="32"/>
-      <c r="O15" s="32"/>
-      <c r="P15" s="32"/>
+      <c r="M15" s="83"/>
+      <c r="N15" s="83"/>
+      <c r="O15" s="83"/>
+      <c r="P15" s="83"/>
       <c r="Q15" s="11"/>
-      <c r="R15" s="33" t="s">
+      <c r="R15" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="S15" s="33"/>
-      <c r="T15" s="33"/>
-      <c r="U15" s="33"/>
-      <c r="V15" s="33"/>
-      <c r="W15" s="33"/>
+      <c r="S15" s="84"/>
+      <c r="T15" s="84"/>
+      <c r="U15" s="84"/>
+      <c r="V15" s="84"/>
+      <c r="W15" s="84"/>
     </row>
-    <row r="16" spans="2:27" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:27" ht="25.5" customHeight="1">
       <c r="B16" s="10"/>
-      <c r="C16" s="34" t="s">
+      <c r="C16" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="34"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="85"/>
+      <c r="F16" s="85"/>
+      <c r="G16" s="85"/>
+      <c r="H16" s="85"/>
+      <c r="I16" s="85"/>
+      <c r="J16" s="85"/>
       <c r="K16" s="9"/>
-      <c r="L16" s="34" t="s">
+      <c r="L16" s="85" t="s">
         <v>43</v>
       </c>
-      <c r="M16" s="35"/>
-      <c r="N16" s="35"/>
-      <c r="O16" s="35"/>
-      <c r="P16" s="35"/>
+      <c r="M16" s="86"/>
+      <c r="N16" s="86"/>
+      <c r="O16" s="86"/>
+      <c r="P16" s="86"/>
       <c r="Q16" s="7"/>
-      <c r="R16" s="35" t="s">
+      <c r="R16" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="S16" s="35"/>
-      <c r="T16" s="35"/>
-      <c r="U16" s="35"/>
-      <c r="V16" s="35"/>
-      <c r="W16" s="35"/>
+      <c r="S16" s="86"/>
+      <c r="T16" s="86"/>
+      <c r="U16" s="86"/>
+      <c r="V16" s="86"/>
+      <c r="W16" s="86"/>
     </row>
-    <row r="17" spans="2:24" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:24" ht="25.5" customHeight="1">
       <c r="B17" s="10"/>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
@@ -3624,7 +3624,7 @@
       <c r="V17" s="6"/>
       <c r="W17" s="6"/>
     </row>
-    <row r="18" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:24" ht="12.75" customHeight="1">
       <c r="B18" s="10"/>
       <c r="C18" s="8"/>
       <c r="D18" s="6"/>
@@ -3648,34 +3648,34 @@
       <c r="V18" s="6"/>
       <c r="W18" s="6"/>
     </row>
-    <row r="19" spans="2:24" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:24" ht="57" customHeight="1">
       <c r="B19" s="4"/>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
-      <c r="J19" s="29"/>
-      <c r="K19" s="29"/>
-      <c r="L19" s="29"/>
-      <c r="M19" s="29"/>
-      <c r="N19" s="29"/>
-      <c r="O19" s="29"/>
-      <c r="P19" s="29"/>
-      <c r="Q19" s="29"/>
-      <c r="R19" s="29"/>
-      <c r="S19" s="29"/>
-      <c r="T19" s="29"/>
-      <c r="U19" s="29"/>
-      <c r="V19" s="29"/>
-      <c r="W19" s="29"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="39"/>
+      <c r="I19" s="39"/>
+      <c r="J19" s="39"/>
+      <c r="K19" s="39"/>
+      <c r="L19" s="39"/>
+      <c r="M19" s="39"/>
+      <c r="N19" s="39"/>
+      <c r="O19" s="39"/>
+      <c r="P19" s="39"/>
+      <c r="Q19" s="39"/>
+      <c r="R19" s="39"/>
+      <c r="S19" s="39"/>
+      <c r="T19" s="39"/>
+      <c r="U19" s="39"/>
+      <c r="V19" s="39"/>
+      <c r="W19" s="39"/>
       <c r="X19" s="4"/>
     </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:24">
       <c r="C21" s="3"/>
       <c r="E21" s="2">
         <v>46176.954704459997</v>
@@ -3683,33 +3683,13 @@
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="C3:J3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="T3:W3"/>
-    <mergeCell ref="P3:R3"/>
-    <mergeCell ref="B1:W1"/>
-    <mergeCell ref="C2:J2"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="T2:W2"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="H4:R4"/>
-    <mergeCell ref="T4:W4"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="H5:R5"/>
-    <mergeCell ref="T5:W5"/>
-    <mergeCell ref="C7:D9"/>
-    <mergeCell ref="E7:M7"/>
-    <mergeCell ref="N7:P9"/>
-    <mergeCell ref="Q7:Q9"/>
-    <mergeCell ref="R7:R9"/>
-    <mergeCell ref="U7:U9"/>
-    <mergeCell ref="V7:V9"/>
-    <mergeCell ref="W7:W9"/>
-    <mergeCell ref="G8:M8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:M9"/>
-    <mergeCell ref="S7:T9"/>
+    <mergeCell ref="C19:W19"/>
+    <mergeCell ref="C13:W13"/>
+    <mergeCell ref="L15:P15"/>
+    <mergeCell ref="R15:W15"/>
+    <mergeCell ref="C16:J16"/>
+    <mergeCell ref="L16:P16"/>
+    <mergeCell ref="R16:W16"/>
     <mergeCell ref="I10:M10"/>
     <mergeCell ref="N10:P10"/>
     <mergeCell ref="S10:T10"/>
@@ -3721,13 +3701,33 @@
     <mergeCell ref="T11:V11"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="G10:H10"/>
-    <mergeCell ref="C19:W19"/>
-    <mergeCell ref="C13:W13"/>
-    <mergeCell ref="L15:P15"/>
-    <mergeCell ref="R15:W15"/>
-    <mergeCell ref="C16:J16"/>
-    <mergeCell ref="L16:P16"/>
-    <mergeCell ref="R16:W16"/>
+    <mergeCell ref="U7:U9"/>
+    <mergeCell ref="V7:V9"/>
+    <mergeCell ref="W7:W9"/>
+    <mergeCell ref="G8:M8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="I9:M9"/>
+    <mergeCell ref="S7:T9"/>
+    <mergeCell ref="C7:D9"/>
+    <mergeCell ref="E7:M7"/>
+    <mergeCell ref="N7:P9"/>
+    <mergeCell ref="Q7:Q9"/>
+    <mergeCell ref="R7:R9"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="H4:R4"/>
+    <mergeCell ref="T4:W4"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="H5:R5"/>
+    <mergeCell ref="T5:W5"/>
+    <mergeCell ref="C3:J3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="T3:W3"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="B1:W1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="T2:W2"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="74" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>

<commit_message>
cambios en el formato y mejoras al editar
</commit_message>
<xml_diff>
--- a/FORMATO.xlsx
+++ b/FORMATO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mauro\Downloads\control-de-clc-y-catálogos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F858BB-8330-44DB-9F00-B5A46275DBC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E78255BF-ED32-47AC-8F8F-7F987A2884F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{83DBF909-10FB-4009-B309-0B7594E05070}"/>
   </bookViews>
@@ -648,7 +648,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -683,10 +683,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -729,6 +725,153 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="6"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -747,12 +890,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="16" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -763,148 +900,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="6"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3099,506 +3098,506 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:27" ht="95.4" customHeight="1">
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
-      <c r="P1" s="39"/>
-      <c r="Q1" s="39"/>
-      <c r="R1" s="39"/>
-      <c r="S1" s="39"/>
-      <c r="T1" s="39"/>
-      <c r="U1" s="39"/>
-      <c r="V1" s="39"/>
-      <c r="W1" s="39"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
       <c r="X1" s="5"/>
-      <c r="AA1" s="25"/>
+      <c r="AA1" s="23"/>
     </row>
     <row r="2" spans="2:27" ht="15.75" customHeight="1">
       <c r="B2" s="5"/>
-      <c r="C2" s="40" t="s">
+      <c r="C2" s="84" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="24"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="84"/>
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="22"/>
       <c r="L2" s="5"/>
-      <c r="M2" s="40" t="s">
+      <c r="M2" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="40"/>
+      <c r="N2" s="84"/>
       <c r="O2" s="5"/>
-      <c r="P2" s="41" t="s">
+      <c r="P2" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="42"/>
       <c r="S2" s="5"/>
-      <c r="T2" s="40" t="s">
+      <c r="T2" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="U2" s="40"/>
-      <c r="V2" s="40"/>
-      <c r="W2" s="40"/>
+      <c r="U2" s="84"/>
+      <c r="V2" s="84"/>
+      <c r="W2" s="84"/>
       <c r="X2" s="5"/>
     </row>
     <row r="3" spans="2:27" ht="27.75" customHeight="1">
-      <c r="B3" s="19"/>
-      <c r="C3" s="28" t="s">
+      <c r="B3" s="17"/>
+      <c r="C3" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="23"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="31" t="s">
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="77"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="17"/>
+      <c r="M3" s="78" t="s">
         <v>29</v>
       </c>
-      <c r="N3" s="32"/>
+      <c r="N3" s="79"/>
       <c r="O3" s="10"/>
-      <c r="P3" s="36" t="s">
+      <c r="P3" s="81" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" s="37"/>
-      <c r="R3" s="38"/>
+      <c r="Q3" s="82"/>
+      <c r="R3" s="83"/>
       <c r="S3" s="10"/>
-      <c r="T3" s="33" t="s">
+      <c r="T3" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="34"/>
-      <c r="V3" s="34"/>
-      <c r="W3" s="35"/>
-      <c r="X3" s="19"/>
+      <c r="U3" s="73"/>
+      <c r="V3" s="73"/>
+      <c r="W3" s="74"/>
+      <c r="X3" s="17"/>
     </row>
     <row r="4" spans="2:27" ht="22.5" customHeight="1">
       <c r="B4" s="10"/>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
       <c r="G4" s="10"/>
-      <c r="H4" s="42" t="s">
+      <c r="H4" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="42"/>
-      <c r="J4" s="42"/>
-      <c r="K4" s="42"/>
-      <c r="L4" s="42"/>
-      <c r="M4" s="42"/>
-      <c r="N4" s="42"/>
-      <c r="O4" s="42"/>
-      <c r="P4" s="42"/>
-      <c r="Q4" s="42"/>
-      <c r="R4" s="42"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="68"/>
+      <c r="O4" s="68"/>
+      <c r="P4" s="68"/>
+      <c r="Q4" s="68"/>
+      <c r="R4" s="68"/>
       <c r="S4" s="10"/>
-      <c r="T4" s="42" t="s">
+      <c r="T4" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="U4" s="42"/>
-      <c r="V4" s="42"/>
-      <c r="W4" s="42"/>
+      <c r="U4" s="68"/>
+      <c r="V4" s="68"/>
+      <c r="W4" s="68"/>
       <c r="X4" s="10"/>
     </row>
     <row r="5" spans="2:27" ht="25.5" customHeight="1">
-      <c r="B5" s="19"/>
-      <c r="C5" s="43" t="s">
+      <c r="B5" s="17"/>
+      <c r="C5" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="46" t="s">
+      <c r="D5" s="70"/>
+      <c r="E5" s="70"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="72" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="34"/>
-      <c r="N5" s="34"/>
-      <c r="O5" s="34"/>
-      <c r="P5" s="34"/>
-      <c r="Q5" s="34"/>
-      <c r="R5" s="35"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="46" t="s">
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
+      <c r="L5" s="73"/>
+      <c r="M5" s="73"/>
+      <c r="N5" s="73"/>
+      <c r="O5" s="73"/>
+      <c r="P5" s="73"/>
+      <c r="Q5" s="73"/>
+      <c r="R5" s="74"/>
+      <c r="S5" s="17"/>
+      <c r="T5" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="U5" s="34"/>
-      <c r="V5" s="34"/>
-      <c r="W5" s="35"/>
-      <c r="X5" s="19"/>
+      <c r="U5" s="73"/>
+      <c r="V5" s="73"/>
+      <c r="W5" s="74"/>
+      <c r="X5" s="17"/>
     </row>
     <row r="6" spans="2:27" ht="17.25" customHeight="1">
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
-      <c r="P6" s="19"/>
-      <c r="Q6" s="19"/>
-      <c r="R6" s="19"/>
-      <c r="S6" s="19"/>
-      <c r="T6" s="19"/>
-      <c r="U6" s="19"/>
-      <c r="V6" s="19"/>
-      <c r="W6" s="19"/>
-      <c r="X6" s="19"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="17"/>
+      <c r="U6" s="17"/>
+      <c r="V6" s="17"/>
+      <c r="W6" s="17"/>
+      <c r="X6" s="17"/>
     </row>
     <row r="7" spans="2:27" ht="12.75" customHeight="1">
-      <c r="B7" s="19"/>
-      <c r="C7" s="47" t="s">
+      <c r="B7" s="17"/>
+      <c r="C7" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="48"/>
-      <c r="E7" s="51" t="s">
+      <c r="D7" s="54"/>
+      <c r="E7" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="52"/>
-      <c r="G7" s="52"/>
-      <c r="H7" s="52"/>
-      <c r="I7" s="52"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="52"/>
-      <c r="L7" s="52"/>
-      <c r="M7" s="53"/>
-      <c r="N7" s="54" t="s">
+      <c r="F7" s="51"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="51"/>
+      <c r="I7" s="51"/>
+      <c r="J7" s="51"/>
+      <c r="K7" s="51"/>
+      <c r="L7" s="51"/>
+      <c r="M7" s="52"/>
+      <c r="N7" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="55"/>
-      <c r="P7" s="56"/>
-      <c r="Q7" s="63" t="s">
+      <c r="O7" s="60"/>
+      <c r="P7" s="61"/>
+      <c r="Q7" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="R7" s="63" t="s">
+      <c r="R7" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="S7" s="66" t="s">
+      <c r="S7" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="T7" s="48"/>
-      <c r="U7" s="63" t="s">
+      <c r="T7" s="54"/>
+      <c r="U7" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="V7" s="63" t="s">
+      <c r="V7" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="W7" s="63" t="s">
+      <c r="W7" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="X7" s="19"/>
+      <c r="X7" s="17"/>
     </row>
     <row r="8" spans="2:27" ht="15" customHeight="1">
       <c r="B8" s="10"/>
-      <c r="C8" s="49"/>
-      <c r="D8" s="50"/>
-      <c r="E8" s="27" t="s">
+      <c r="C8" s="57"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="27" t="s">
+      <c r="F8" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="51" t="s">
+      <c r="G8" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="52"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="52"/>
-      <c r="L8" s="52"/>
-      <c r="M8" s="53"/>
-      <c r="N8" s="57"/>
-      <c r="O8" s="58"/>
-      <c r="P8" s="59"/>
-      <c r="Q8" s="64"/>
-      <c r="R8" s="64"/>
-      <c r="S8" s="49"/>
-      <c r="T8" s="50"/>
-      <c r="U8" s="64"/>
-      <c r="V8" s="64"/>
-      <c r="W8" s="64"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="51"/>
+      <c r="J8" s="51"/>
+      <c r="K8" s="51"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="52"/>
+      <c r="N8" s="62"/>
+      <c r="O8" s="63"/>
+      <c r="P8" s="64"/>
+      <c r="Q8" s="49"/>
+      <c r="R8" s="49"/>
+      <c r="S8" s="57"/>
+      <c r="T8" s="58"/>
+      <c r="U8" s="49"/>
+      <c r="V8" s="49"/>
+      <c r="W8" s="49"/>
       <c r="X8" s="10"/>
     </row>
     <row r="9" spans="2:27" ht="20.25" customHeight="1">
-      <c r="B9" s="19"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="26" t="s">
+      <c r="B9" s="17"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="26" t="s">
+      <c r="F9" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="47" t="s">
+      <c r="G9" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="48"/>
-      <c r="I9" s="47" t="s">
+      <c r="H9" s="54"/>
+      <c r="I9" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="J9" s="65"/>
-      <c r="K9" s="65"/>
-      <c r="L9" s="65"/>
-      <c r="M9" s="48"/>
-      <c r="N9" s="60"/>
-      <c r="O9" s="61"/>
-      <c r="P9" s="62"/>
-      <c r="Q9" s="64"/>
-      <c r="R9" s="64"/>
-      <c r="S9" s="49"/>
-      <c r="T9" s="50"/>
-      <c r="U9" s="64"/>
-      <c r="V9" s="64"/>
-      <c r="W9" s="64"/>
-      <c r="X9" s="19"/>
+      <c r="J9" s="55"/>
+      <c r="K9" s="55"/>
+      <c r="L9" s="55"/>
+      <c r="M9" s="54"/>
+      <c r="N9" s="65"/>
+      <c r="O9" s="66"/>
+      <c r="P9" s="67"/>
+      <c r="Q9" s="49"/>
+      <c r="R9" s="49"/>
+      <c r="S9" s="57"/>
+      <c r="T9" s="58"/>
+      <c r="U9" s="49"/>
+      <c r="V9" s="49"/>
+      <c r="W9" s="49"/>
+      <c r="X9" s="17"/>
     </row>
     <row r="10" spans="2:27" ht="59.25" customHeight="1">
-      <c r="B10" s="19"/>
-      <c r="C10" s="79">
+      <c r="B10" s="17"/>
+      <c r="C10" s="47">
         <v>4446</v>
       </c>
-      <c r="D10" s="79"/>
-      <c r="E10" s="22" t="s">
+      <c r="D10" s="47"/>
+      <c r="E10" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="F10" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="67" t="s">
+      <c r="G10" s="34" t="s">
         <v>37</v>
       </c>
-      <c r="H10" s="67"/>
-      <c r="I10" s="67" t="s">
+      <c r="H10" s="34"/>
+      <c r="I10" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="67"/>
-      <c r="K10" s="67"/>
-      <c r="L10" s="67"/>
-      <c r="M10" s="67"/>
-      <c r="N10" s="68" t="s">
+      <c r="J10" s="34"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="O10" s="69"/>
-      <c r="P10" s="70"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="20">
+      <c r="O10" s="36"/>
+      <c r="P10" s="37"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="18">
         <v>1</v>
       </c>
-      <c r="S10" s="71">
+      <c r="S10" s="38">
         <v>0</v>
       </c>
-      <c r="T10" s="72"/>
-      <c r="U10" s="20">
+      <c r="T10" s="39"/>
+      <c r="U10" s="18">
         <v>0.16</v>
       </c>
-      <c r="V10" s="20">
+      <c r="V10" s="18">
         <v>0</v>
       </c>
-      <c r="W10" s="20">
+      <c r="W10" s="18">
         <f>R10-S10+U10-V10</f>
         <v>1.1599999999999999</v>
       </c>
-      <c r="X10" s="19"/>
+      <c r="X10" s="17"/>
     </row>
-    <row r="11" spans="2:27" s="14" customFormat="1" ht="48.75" customHeight="1">
+    <row r="11" spans="2:27" s="12" customFormat="1" ht="48.75" customHeight="1">
       <c r="B11" s="10"/>
-      <c r="C11" s="75" t="s">
+      <c r="C11" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="76"/>
-      <c r="E11" s="76"/>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="76"/>
-      <c r="I11" s="76"/>
-      <c r="J11" s="76"/>
-      <c r="K11" s="76"/>
-      <c r="L11" s="76"/>
-      <c r="M11" s="76"/>
-      <c r="N11" s="76"/>
-      <c r="O11" s="76"/>
-      <c r="P11" s="76"/>
-      <c r="Q11" s="76"/>
-      <c r="R11" s="76"/>
-      <c r="S11" s="77"/>
-      <c r="T11" s="78" t="s">
+      <c r="D11" s="44"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="44"/>
+      <c r="M11" s="44"/>
+      <c r="N11" s="44"/>
+      <c r="O11" s="44"/>
+      <c r="P11" s="44"/>
+      <c r="Q11" s="44"/>
+      <c r="R11" s="44"/>
+      <c r="S11" s="45"/>
+      <c r="T11" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="U11" s="78"/>
-      <c r="V11" s="78"/>
-      <c r="W11" s="15">
+      <c r="U11" s="46"/>
+      <c r="V11" s="46"/>
+      <c r="W11" s="13">
         <f>SUM(W10:W10)</f>
         <v>1.1599999999999999</v>
       </c>
       <c r="X11" s="10"/>
     </row>
-    <row r="12" spans="2:27" s="14" customFormat="1" ht="14.25" customHeight="1">
+    <row r="12" spans="2:27" s="12" customFormat="1" ht="14.25" customHeight="1">
       <c r="B12" s="10"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-      <c r="O12" s="18"/>
-      <c r="P12" s="18"/>
-      <c r="Q12" s="18"/>
-      <c r="R12" s="18"/>
-      <c r="S12" s="17"/>
-      <c r="T12" s="16"/>
-      <c r="U12" s="16"/>
-      <c r="V12" s="16"/>
-      <c r="W12" s="15"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="16"/>
+      <c r="P12" s="16"/>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="16"/>
+      <c r="S12" s="15"/>
+      <c r="T12" s="14"/>
+      <c r="U12" s="14"/>
+      <c r="V12" s="14"/>
+      <c r="W12" s="13"/>
       <c r="X12" s="10"/>
     </row>
     <row r="13" spans="2:27" ht="12" customHeight="1">
-      <c r="C13" s="81"/>
-      <c r="D13" s="82"/>
-      <c r="E13" s="82"/>
-      <c r="F13" s="82"/>
-      <c r="G13" s="82"/>
-      <c r="H13" s="82"/>
-      <c r="I13" s="82"/>
-      <c r="J13" s="82"/>
-      <c r="K13" s="82"/>
-      <c r="L13" s="82"/>
-      <c r="M13" s="82"/>
-      <c r="N13" s="82"/>
-      <c r="O13" s="82"/>
-      <c r="P13" s="82"/>
-      <c r="Q13" s="82"/>
-      <c r="R13" s="82"/>
-      <c r="S13" s="82"/>
-      <c r="T13" s="82"/>
-      <c r="U13" s="82"/>
-      <c r="V13" s="82"/>
-      <c r="W13" s="82"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+      <c r="J13" s="29"/>
+      <c r="K13" s="29"/>
+      <c r="L13" s="29"/>
+      <c r="M13" s="29"/>
+      <c r="N13" s="29"/>
+      <c r="O13" s="29"/>
+      <c r="P13" s="29"/>
+      <c r="Q13" s="29"/>
+      <c r="R13" s="29"/>
+      <c r="S13" s="29"/>
+      <c r="T13" s="29"/>
+      <c r="U13" s="29"/>
+      <c r="V13" s="29"/>
+      <c r="W13" s="29"/>
       <c r="X13" s="4"/>
-      <c r="Y13" s="73"/>
-      <c r="Z13" s="73"/>
+      <c r="Y13" s="40"/>
+      <c r="Z13" s="40"/>
     </row>
     <row r="14" spans="2:27" ht="12.75" customHeight="1">
-      <c r="C14" s="74" t="s">
+      <c r="C14" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="41"/>
-      <c r="I14" s="41"/>
-      <c r="L14" s="74" t="s">
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="42"/>
+      <c r="L14" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="M14" s="41"/>
-      <c r="N14" s="41"/>
-      <c r="O14" s="41"/>
-      <c r="P14" s="41"/>
-      <c r="R14" s="74" t="s">
+      <c r="M14" s="42"/>
+      <c r="N14" s="42"/>
+      <c r="O14" s="42"/>
+      <c r="P14" s="42"/>
+      <c r="R14" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="S14" s="41"/>
-      <c r="T14" s="41"/>
-      <c r="U14" s="41"/>
-      <c r="V14" s="41"/>
-      <c r="W14" s="41"/>
+      <c r="S14" s="42"/>
+      <c r="T14" s="42"/>
+      <c r="U14" s="42"/>
+      <c r="V14" s="42"/>
+      <c r="W14" s="42"/>
     </row>
     <row r="15" spans="2:27" ht="76.5" customHeight="1">
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="85" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="12"/>
+      <c r="D15" s="85"/>
+      <c r="E15" s="85"/>
+      <c r="F15" s="85"/>
+      <c r="G15" s="85"/>
+      <c r="H15" s="85"/>
+      <c r="I15" s="85"/>
+      <c r="J15" s="85"/>
       <c r="K15" s="9"/>
-      <c r="L15" s="83" t="s">
+      <c r="L15" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="M15" s="83"/>
-      <c r="N15" s="83"/>
-      <c r="O15" s="83"/>
-      <c r="P15" s="83"/>
+      <c r="M15" s="30"/>
+      <c r="N15" s="30"/>
+      <c r="O15" s="30"/>
+      <c r="P15" s="30"/>
       <c r="Q15" s="11"/>
-      <c r="R15" s="84" t="s">
+      <c r="R15" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="S15" s="84"/>
-      <c r="T15" s="84"/>
-      <c r="U15" s="84"/>
-      <c r="V15" s="84"/>
-      <c r="W15" s="84"/>
+      <c r="S15" s="31"/>
+      <c r="T15" s="31"/>
+      <c r="U15" s="31"/>
+      <c r="V15" s="31"/>
+      <c r="W15" s="31"/>
     </row>
     <row r="16" spans="2:27" ht="25.5" customHeight="1">
       <c r="B16" s="10"/>
-      <c r="C16" s="85" t="s">
+      <c r="C16" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="85"/>
-      <c r="E16" s="85"/>
-      <c r="F16" s="85"/>
-      <c r="G16" s="85"/>
-      <c r="H16" s="85"/>
-      <c r="I16" s="85"/>
-      <c r="J16" s="85"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
       <c r="K16" s="9"/>
-      <c r="L16" s="85" t="s">
+      <c r="L16" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="M16" s="86"/>
-      <c r="N16" s="86"/>
-      <c r="O16" s="86"/>
-      <c r="P16" s="86"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="33"/>
+      <c r="P16" s="33"/>
       <c r="Q16" s="7"/>
-      <c r="R16" s="86" t="s">
+      <c r="R16" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="S16" s="86"/>
-      <c r="T16" s="86"/>
-      <c r="U16" s="86"/>
-      <c r="V16" s="86"/>
-      <c r="W16" s="86"/>
+      <c r="S16" s="33"/>
+      <c r="T16" s="33"/>
+      <c r="U16" s="33"/>
+      <c r="V16" s="33"/>
+      <c r="W16" s="33"/>
     </row>
     <row r="17" spans="2:24" ht="25.5" customHeight="1">
       <c r="B17" s="10"/>
@@ -3650,29 +3649,29 @@
     </row>
     <row r="19" spans="2:24" ht="57" customHeight="1">
       <c r="B19" s="4"/>
-      <c r="C19" s="80" t="s">
+      <c r="C19" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="39"/>
-      <c r="I19" s="39"/>
-      <c r="J19" s="39"/>
-      <c r="K19" s="39"/>
-      <c r="L19" s="39"/>
-      <c r="M19" s="39"/>
-      <c r="N19" s="39"/>
-      <c r="O19" s="39"/>
-      <c r="P19" s="39"/>
-      <c r="Q19" s="39"/>
-      <c r="R19" s="39"/>
-      <c r="S19" s="39"/>
-      <c r="T19" s="39"/>
-      <c r="U19" s="39"/>
-      <c r="V19" s="39"/>
-      <c r="W19" s="39"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="27"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="27"/>
+      <c r="P19" s="27"/>
+      <c r="Q19" s="27"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="27"/>
+      <c r="U19" s="27"/>
+      <c r="V19" s="27"/>
+      <c r="W19" s="27"/>
       <c r="X19" s="4"/>
     </row>
     <row r="21" spans="2:24">
@@ -3682,14 +3681,34 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="45">
-    <mergeCell ref="C19:W19"/>
-    <mergeCell ref="C13:W13"/>
-    <mergeCell ref="L15:P15"/>
-    <mergeCell ref="R15:W15"/>
-    <mergeCell ref="C16:J16"/>
-    <mergeCell ref="L16:P16"/>
-    <mergeCell ref="R16:W16"/>
+  <mergeCells count="46">
+    <mergeCell ref="C3:J3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="T3:W3"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="B1:W1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="T2:W2"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="H4:R4"/>
+    <mergeCell ref="T4:W4"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="H5:R5"/>
+    <mergeCell ref="T5:W5"/>
+    <mergeCell ref="C7:D9"/>
+    <mergeCell ref="E7:M7"/>
+    <mergeCell ref="N7:P9"/>
+    <mergeCell ref="Q7:Q9"/>
+    <mergeCell ref="R7:R9"/>
+    <mergeCell ref="U7:U9"/>
+    <mergeCell ref="V7:V9"/>
+    <mergeCell ref="W7:W9"/>
+    <mergeCell ref="G8:M8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="I9:M9"/>
+    <mergeCell ref="S7:T9"/>
     <mergeCell ref="I10:M10"/>
     <mergeCell ref="N10:P10"/>
     <mergeCell ref="S10:T10"/>
@@ -3701,33 +3720,14 @@
     <mergeCell ref="T11:V11"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="G10:H10"/>
-    <mergeCell ref="U7:U9"/>
-    <mergeCell ref="V7:V9"/>
-    <mergeCell ref="W7:W9"/>
-    <mergeCell ref="G8:M8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:M9"/>
-    <mergeCell ref="S7:T9"/>
-    <mergeCell ref="C7:D9"/>
-    <mergeCell ref="E7:M7"/>
-    <mergeCell ref="N7:P9"/>
-    <mergeCell ref="Q7:Q9"/>
-    <mergeCell ref="R7:R9"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="H4:R4"/>
-    <mergeCell ref="T4:W4"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="H5:R5"/>
-    <mergeCell ref="T5:W5"/>
-    <mergeCell ref="C3:J3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="T3:W3"/>
-    <mergeCell ref="P3:R3"/>
-    <mergeCell ref="B1:W1"/>
-    <mergeCell ref="C2:J2"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="T2:W2"/>
+    <mergeCell ref="C19:W19"/>
+    <mergeCell ref="C13:W13"/>
+    <mergeCell ref="L15:P15"/>
+    <mergeCell ref="R15:W15"/>
+    <mergeCell ref="C16:J16"/>
+    <mergeCell ref="L16:P16"/>
+    <mergeCell ref="R16:W16"/>
+    <mergeCell ref="C15:J15"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="74" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>